<commit_message>
feat(lac): South Asia's loss rule and A settings with the floor top-up
- setup.yaml: policy apply_internal_tx_losses.
- Config_country_codes.yaml: internal_transmission.transmission_loss 0.03
  (ASSUMPTION, uniform across the 19 countries).
- Root workbooks: internal-family input ratios set to 1 in both
  activity-ratio workbooks; Measured_at column on Demand_Projection,
  bus-bar on all 19 demand rows.
- A and C: South Asia A's build-cap settings plus floor_top_up, in place of
  the cap multiplier 0 and the 25 open-capped technologies.
- B: South Asia B's storage exemptions in place of the 25 technologies, plus
  floor_top_up.
</commit_message>
<xml_diff>
--- a/areas/lac/inputs/scenarios/root_workbooks/A-O_AR_Model_Base_Year.xlsx
+++ b/areas/lac/inputs/scenarios/root_workbooks/A-O_AR_Model_Base_Year.xlsx
@@ -33814,7 +33814,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1.006</v>
+        <v>1</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -33855,7 +33855,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1.006</v>
+        <v>1</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -33896,7 +33896,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1.006</v>
+        <v>1</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -33937,7 +33937,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1.005</v>
+        <v>1</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -33978,7 +33978,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1.006</v>
+        <v>1</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -34019,7 +34019,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1.005</v>
+        <v>1</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -34142,7 +34142,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>1.031</v>
+        <v>1</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -34183,7 +34183,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>1.031</v>
+        <v>1</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -34224,7 +34224,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>1.031</v>
+        <v>1</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -34265,7 +34265,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>1.02</v>
+        <v>1</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -34306,7 +34306,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>1.031</v>
+        <v>1</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -34347,7 +34347,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>1.02</v>
+        <v>1</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -34470,7 +34470,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>1.037</v>
+        <v>1</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -34511,7 +34511,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>1.037</v>
+        <v>1</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -34552,7 +34552,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>1.037</v>
+        <v>1</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -34593,7 +34593,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>1.01</v>
+        <v>1</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -34634,7 +34634,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>1.037</v>
+        <v>1</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
@@ -34675,7 +34675,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>1.01</v>
+        <v>1</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -34798,7 +34798,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>1.033</v>
+        <v>1</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -34839,7 +34839,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>1.033</v>
+        <v>1</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -34880,7 +34880,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>1.033</v>
+        <v>1</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -34921,7 +34921,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>1.008</v>
+        <v>1</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
@@ -34962,7 +34962,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>1.033</v>
+        <v>1</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
@@ -35003,7 +35003,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>1.008</v>
+        <v>1</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
@@ -35126,7 +35126,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>1.031</v>
+        <v>1</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
@@ -35167,7 +35167,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>1.031</v>
+        <v>1</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
@@ -35208,7 +35208,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>1.031</v>
+        <v>1</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
@@ -35249,7 +35249,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>1.01</v>
+        <v>1</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
@@ -35290,7 +35290,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>1.031</v>
+        <v>1</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
@@ -35331,7 +35331,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>1.01</v>
+        <v>1</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
@@ -35454,7 +35454,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>1.034</v>
+        <v>1</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
@@ -35495,7 +35495,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>1.034</v>
+        <v>1</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
@@ -35536,7 +35536,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>1.034</v>
+        <v>1</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
@@ -35577,7 +35577,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>1.02</v>
+        <v>1</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
@@ -35618,7 +35618,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>1.034</v>
+        <v>1</v>
       </c>
       <c r="F46" t="inlineStr">
         <is>
@@ -35659,7 +35659,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>1.02</v>
+        <v>1</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
@@ -35782,7 +35782,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>1.015</v>
+        <v>1</v>
       </c>
       <c r="F50" t="inlineStr">
         <is>
@@ -35823,7 +35823,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>1.015</v>
+        <v>1</v>
       </c>
       <c r="F51" t="inlineStr">
         <is>
@@ -35864,7 +35864,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>1.015</v>
+        <v>1</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
@@ -35905,7 +35905,7 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>1.006</v>
+        <v>1</v>
       </c>
       <c r="F53" t="inlineStr">
         <is>
@@ -35946,7 +35946,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>1.015</v>
+        <v>1</v>
       </c>
       <c r="F54" t="inlineStr">
         <is>
@@ -35987,7 +35987,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>1.006</v>
+        <v>1</v>
       </c>
       <c r="F55" t="inlineStr">
         <is>
@@ -36110,7 +36110,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>1.026</v>
+        <v>1</v>
       </c>
       <c r="F58" t="inlineStr">
         <is>
@@ -36151,7 +36151,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>1.026</v>
+        <v>1</v>
       </c>
       <c r="F59" t="inlineStr">
         <is>
@@ -36192,7 +36192,7 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>1.026</v>
+        <v>1</v>
       </c>
       <c r="F60" t="inlineStr">
         <is>
@@ -36233,7 +36233,7 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>1.013</v>
+        <v>1</v>
       </c>
       <c r="F61" t="inlineStr">
         <is>
@@ -36274,7 +36274,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>1.026</v>
+        <v>1</v>
       </c>
       <c r="F62" t="inlineStr">
         <is>
@@ -36315,7 +36315,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>1.013</v>
+        <v>1</v>
       </c>
       <c r="F63" t="inlineStr">
         <is>
@@ -36438,7 +36438,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>1.018</v>
+        <v>1</v>
       </c>
       <c r="F66" t="inlineStr">
         <is>
@@ -36479,7 +36479,7 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>1.018</v>
+        <v>1</v>
       </c>
       <c r="F67" t="inlineStr">
         <is>
@@ -36520,7 +36520,7 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>1.018</v>
+        <v>1</v>
       </c>
       <c r="F68" t="inlineStr">
         <is>
@@ -36561,7 +36561,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>1.009</v>
+        <v>1</v>
       </c>
       <c r="F69" t="inlineStr">
         <is>
@@ -36602,7 +36602,7 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>1.018</v>
+        <v>1</v>
       </c>
       <c r="F70" t="inlineStr">
         <is>
@@ -36643,7 +36643,7 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>1.009</v>
+        <v>1</v>
       </c>
       <c r="F71" t="inlineStr">
         <is>
@@ -36766,7 +36766,7 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>1.026</v>
+        <v>1</v>
       </c>
       <c r="F74" t="inlineStr">
         <is>
@@ -36807,7 +36807,7 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>1.026</v>
+        <v>1</v>
       </c>
       <c r="F75" t="inlineStr">
         <is>
@@ -36848,7 +36848,7 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>1.026</v>
+        <v>1</v>
       </c>
       <c r="F76" t="inlineStr">
         <is>
@@ -36889,7 +36889,7 @@
         </is>
       </c>
       <c r="D77" t="n">
-        <v>1.015</v>
+        <v>1</v>
       </c>
       <c r="F77" t="inlineStr">
         <is>
@@ -36930,7 +36930,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>1.026</v>
+        <v>1</v>
       </c>
       <c r="F78" t="inlineStr">
         <is>
@@ -36971,7 +36971,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>1.015</v>
+        <v>1</v>
       </c>
       <c r="F79" t="inlineStr">
         <is>
@@ -37094,7 +37094,7 @@
         </is>
       </c>
       <c r="D82" t="n">
-        <v>1.02</v>
+        <v>1</v>
       </c>
       <c r="F82" t="inlineStr">
         <is>
@@ -37135,7 +37135,7 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>1.02</v>
+        <v>1</v>
       </c>
       <c r="F83" t="inlineStr">
         <is>
@@ -37176,7 +37176,7 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>1.02</v>
+        <v>1</v>
       </c>
       <c r="F84" t="inlineStr">
         <is>
@@ -37217,7 +37217,7 @@
         </is>
       </c>
       <c r="D85" t="n">
-        <v>1.01</v>
+        <v>1</v>
       </c>
       <c r="F85" t="inlineStr">
         <is>
@@ -37258,7 +37258,7 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>1.02</v>
+        <v>1</v>
       </c>
       <c r="F86" t="inlineStr">
         <is>
@@ -37299,7 +37299,7 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>1.01</v>
+        <v>1</v>
       </c>
       <c r="F87" t="inlineStr">
         <is>
@@ -37422,7 +37422,7 @@
         </is>
       </c>
       <c r="D90" t="n">
-        <v>1.039</v>
+        <v>1</v>
       </c>
       <c r="F90" t="inlineStr">
         <is>
@@ -37463,7 +37463,7 @@
         </is>
       </c>
       <c r="D91" t="n">
-        <v>1.039</v>
+        <v>1</v>
       </c>
       <c r="F91" t="inlineStr">
         <is>
@@ -37504,7 +37504,7 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>1.039</v>
+        <v>1</v>
       </c>
       <c r="F92" t="inlineStr">
         <is>
@@ -37545,7 +37545,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>1.01</v>
+        <v>1</v>
       </c>
       <c r="F93" t="inlineStr">
         <is>
@@ -37586,7 +37586,7 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>1.039</v>
+        <v>1</v>
       </c>
       <c r="F94" t="inlineStr">
         <is>
@@ -37627,7 +37627,7 @@
         </is>
       </c>
       <c r="D95" t="n">
-        <v>1.01</v>
+        <v>1</v>
       </c>
       <c r="F95" t="inlineStr">
         <is>
@@ -37750,7 +37750,7 @@
         </is>
       </c>
       <c r="D98" t="n">
-        <v>1.039</v>
+        <v>1</v>
       </c>
       <c r="F98" t="inlineStr">
         <is>
@@ -37791,7 +37791,7 @@
         </is>
       </c>
       <c r="D99" t="n">
-        <v>1.039</v>
+        <v>1</v>
       </c>
       <c r="F99" t="inlineStr">
         <is>
@@ -37832,7 +37832,7 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>1.039</v>
+        <v>1</v>
       </c>
       <c r="F100" t="inlineStr">
         <is>
@@ -37873,7 +37873,7 @@
         </is>
       </c>
       <c r="D101" t="n">
-        <v>1.013</v>
+        <v>1</v>
       </c>
       <c r="F101" t="inlineStr">
         <is>
@@ -37914,7 +37914,7 @@
         </is>
       </c>
       <c r="D102" t="n">
-        <v>1.039</v>
+        <v>1</v>
       </c>
       <c r="F102" t="inlineStr">
         <is>
@@ -37955,7 +37955,7 @@
         </is>
       </c>
       <c r="D103" t="n">
-        <v>1.013</v>
+        <v>1</v>
       </c>
       <c r="F103" t="inlineStr">
         <is>
@@ -38078,7 +38078,7 @@
         </is>
       </c>
       <c r="D106" t="n">
-        <v>1.029</v>
+        <v>1</v>
       </c>
       <c r="F106" t="inlineStr">
         <is>
@@ -38119,7 +38119,7 @@
         </is>
       </c>
       <c r="D107" t="n">
-        <v>1.029</v>
+        <v>1</v>
       </c>
       <c r="F107" t="inlineStr">
         <is>
@@ -38160,7 +38160,7 @@
         </is>
       </c>
       <c r="D108" t="n">
-        <v>1.029</v>
+        <v>1</v>
       </c>
       <c r="F108" t="inlineStr">
         <is>
@@ -38201,7 +38201,7 @@
         </is>
       </c>
       <c r="D109" t="n">
-        <v>1.006</v>
+        <v>1</v>
       </c>
       <c r="F109" t="inlineStr">
         <is>
@@ -38242,7 +38242,7 @@
         </is>
       </c>
       <c r="D110" t="n">
-        <v>1.029</v>
+        <v>1</v>
       </c>
       <c r="F110" t="inlineStr">
         <is>
@@ -38283,7 +38283,7 @@
         </is>
       </c>
       <c r="D111" t="n">
-        <v>1.006</v>
+        <v>1</v>
       </c>
       <c r="F111" t="inlineStr">
         <is>
@@ -38406,7 +38406,7 @@
         </is>
       </c>
       <c r="D114" t="n">
-        <v>1.033</v>
+        <v>1</v>
       </c>
       <c r="F114" t="inlineStr">
         <is>
@@ -38447,7 +38447,7 @@
         </is>
       </c>
       <c r="D115" t="n">
-        <v>1.033</v>
+        <v>1</v>
       </c>
       <c r="F115" t="inlineStr">
         <is>
@@ -38488,7 +38488,7 @@
         </is>
       </c>
       <c r="D116" t="n">
-        <v>1.033</v>
+        <v>1</v>
       </c>
       <c r="F116" t="inlineStr">
         <is>
@@ -38529,7 +38529,7 @@
         </is>
       </c>
       <c r="D117" t="n">
-        <v>1.016</v>
+        <v>1</v>
       </c>
       <c r="F117" t="inlineStr">
         <is>
@@ -38570,7 +38570,7 @@
         </is>
       </c>
       <c r="D118" t="n">
-        <v>1.033</v>
+        <v>1</v>
       </c>
       <c r="F118" t="inlineStr">
         <is>
@@ -38611,7 +38611,7 @@
         </is>
       </c>
       <c r="D119" t="n">
-        <v>1.016</v>
+        <v>1</v>
       </c>
       <c r="F119" t="inlineStr">
         <is>
@@ -38734,7 +38734,7 @@
         </is>
       </c>
       <c r="D122" t="n">
-        <v>1.016</v>
+        <v>1</v>
       </c>
       <c r="F122" t="inlineStr">
         <is>
@@ -38775,7 +38775,7 @@
         </is>
       </c>
       <c r="D123" t="n">
-        <v>1.016</v>
+        <v>1</v>
       </c>
       <c r="F123" t="inlineStr">
         <is>
@@ -38816,7 +38816,7 @@
         </is>
       </c>
       <c r="D124" t="n">
-        <v>1.016</v>
+        <v>1</v>
       </c>
       <c r="F124" t="inlineStr">
         <is>
@@ -38857,7 +38857,7 @@
         </is>
       </c>
       <c r="D125" t="n">
-        <v>1.003</v>
+        <v>1</v>
       </c>
       <c r="F125" t="inlineStr">
         <is>
@@ -38898,7 +38898,7 @@
         </is>
       </c>
       <c r="D126" t="n">
-        <v>1.016</v>
+        <v>1</v>
       </c>
       <c r="F126" t="inlineStr">
         <is>
@@ -38939,7 +38939,7 @@
         </is>
       </c>
       <c r="D127" t="n">
-        <v>1.003</v>
+        <v>1</v>
       </c>
       <c r="F127" t="inlineStr">
         <is>
@@ -39062,7 +39062,7 @@
         </is>
       </c>
       <c r="D130" t="n">
-        <v>1.05</v>
+        <v>1</v>
       </c>
       <c r="F130" t="inlineStr">
         <is>
@@ -39103,7 +39103,7 @@
         </is>
       </c>
       <c r="D131" t="n">
-        <v>1.05</v>
+        <v>1</v>
       </c>
       <c r="F131" t="inlineStr">
         <is>
@@ -39144,7 +39144,7 @@
         </is>
       </c>
       <c r="D132" t="n">
-        <v>1.05</v>
+        <v>1</v>
       </c>
       <c r="F132" t="inlineStr">
         <is>
@@ -39185,7 +39185,7 @@
         </is>
       </c>
       <c r="D133" t="n">
-        <v>1.012</v>
+        <v>1</v>
       </c>
       <c r="F133" t="inlineStr">
         <is>
@@ -39226,7 +39226,7 @@
         </is>
       </c>
       <c r="D134" t="n">
-        <v>1.05</v>
+        <v>1</v>
       </c>
       <c r="F134" t="inlineStr">
         <is>
@@ -39267,7 +39267,7 @@
         </is>
       </c>
       <c r="D135" t="n">
-        <v>1.012</v>
+        <v>1</v>
       </c>
       <c r="F135" t="inlineStr">
         <is>
@@ -39390,7 +39390,7 @@
         </is>
       </c>
       <c r="D138" t="n">
-        <v>1.044</v>
+        <v>1</v>
       </c>
       <c r="F138" t="inlineStr">
         <is>
@@ -39431,7 +39431,7 @@
         </is>
       </c>
       <c r="D139" t="n">
-        <v>1.044</v>
+        <v>1</v>
       </c>
       <c r="F139" t="inlineStr">
         <is>
@@ -39472,7 +39472,7 @@
         </is>
       </c>
       <c r="D140" t="n">
-        <v>1.044</v>
+        <v>1</v>
       </c>
       <c r="F140" t="inlineStr">
         <is>
@@ -39513,7 +39513,7 @@
         </is>
       </c>
       <c r="D141" t="n">
-        <v>1.025</v>
+        <v>1</v>
       </c>
       <c r="F141" t="inlineStr">
         <is>
@@ -39554,7 +39554,7 @@
         </is>
       </c>
       <c r="D142" t="n">
-        <v>1.044</v>
+        <v>1</v>
       </c>
       <c r="F142" t="inlineStr">
         <is>
@@ -39595,7 +39595,7 @@
         </is>
       </c>
       <c r="D143" t="n">
-        <v>1.025</v>
+        <v>1</v>
       </c>
       <c r="F143" t="inlineStr">
         <is>
@@ -39718,7 +39718,7 @@
         </is>
       </c>
       <c r="D146" t="n">
-        <v>1.042</v>
+        <v>1</v>
       </c>
       <c r="F146" t="inlineStr">
         <is>
@@ -39759,7 +39759,7 @@
         </is>
       </c>
       <c r="D147" t="n">
-        <v>1.042</v>
+        <v>1</v>
       </c>
       <c r="F147" t="inlineStr">
         <is>
@@ -39800,7 +39800,7 @@
         </is>
       </c>
       <c r="D148" t="n">
-        <v>1.042</v>
+        <v>1</v>
       </c>
       <c r="F148" t="inlineStr">
         <is>
@@ -39841,7 +39841,7 @@
         </is>
       </c>
       <c r="D149" t="n">
-        <v>1.012</v>
+        <v>1</v>
       </c>
       <c r="F149" t="inlineStr">
         <is>
@@ -39882,7 +39882,7 @@
         </is>
       </c>
       <c r="D150" t="n">
-        <v>1.042</v>
+        <v>1</v>
       </c>
       <c r="F150" t="inlineStr">
         <is>
@@ -39923,7 +39923,7 @@
         </is>
       </c>
       <c r="D151" t="n">
-        <v>1.012</v>
+        <v>1</v>
       </c>
       <c r="F151" t="inlineStr">
         <is>

</xml_diff>